<commit_message>
archived and recent price history api calls script complete
</commit_message>
<xml_diff>
--- a/electricity/src/hydrate/retail/lmp_territory_assignments.xlsx
+++ b/electricity/src/hydrate/retail/lmp_territory_assignments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\darbvt\spring26\project-spring26-darbyatNE\electricity\src\hydrate\retail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98111E8B-B1F6-44B5-ABA6-5FF8D1E03742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7527BDC1-CE55-406A-B65E-6A1B7C5E3887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapped_LMPs" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6134" uniqueCount="1987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6222" uniqueCount="2017">
   <si>
     <t>Zone</t>
   </si>
@@ -5997,6 +5997,96 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Pike County Light &amp; Power Co</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Milford, PA</t>
+  </si>
+  <si>
+    <t>Bushkill, PA</t>
+  </si>
+  <si>
+    <t>Dingmans Ferry, PA</t>
+  </si>
+  <si>
+    <t>DINGMANS</t>
+  </si>
+  <si>
+    <t>BUSHKILL</t>
+  </si>
+  <si>
+    <t>POCONO</t>
+  </si>
+  <si>
+    <t>BLMG</t>
+  </si>
+  <si>
+    <t>Likely in Pocono area, Pike County or nearby</t>
+  </si>
+  <si>
+    <t>POCONO_F</t>
+  </si>
+  <si>
+    <t>POFA1_LD</t>
+  </si>
+  <si>
+    <t>POFA2_LD</t>
+  </si>
+  <si>
+    <t>MTPOCONO</t>
+  </si>
+  <si>
+    <t>MOPO1_LD</t>
+  </si>
+  <si>
+    <t>Mount Pocono, near Pike County</t>
+  </si>
+  <si>
+    <t>MOPO2_LD</t>
+  </si>
+  <si>
+    <t>HAWLEYPL</t>
+  </si>
+  <si>
+    <t>HAWL_LD</t>
+  </si>
+  <si>
+    <t>Hawley, PA, in Pike County</t>
+  </si>
+  <si>
+    <t>HONSDALE</t>
+  </si>
+  <si>
+    <t>HONE1_LD</t>
+  </si>
+  <si>
+    <t>Honesdale, PA, near Pike County (Wayne County)</t>
+  </si>
+  <si>
+    <t>HONE2_LD</t>
+  </si>
+  <si>
+    <t>KIMBLES</t>
+  </si>
+  <si>
+    <t>KIMB_LD</t>
+  </si>
+  <si>
+    <t>Kimble, PA, in Pike County</t>
+  </si>
+  <si>
+    <t>TAFTON</t>
+  </si>
+  <si>
+    <t>TAFT_LD</t>
+  </si>
+  <si>
+    <t>Tafton, PA, in Pike County</t>
   </si>
 </sst>
 </file>
@@ -6369,13 +6459,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1022"/>
+  <dimension ref="A1:H1035"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -32928,7 +33018,7 @@
         <v>1674</v>
       </c>
     </row>
-    <row r="1022" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1022" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1022" t="s">
         <v>456</v>
       </c>
@@ -32952,6 +33042,314 @@
       </c>
       <c r="H1022" t="s">
         <v>1834</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1023" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1023" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1023" s="2" t="s">
+        <v>1559</v>
+      </c>
+      <c r="D1023" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1023" s="2" t="s">
+        <v>1988</v>
+      </c>
+      <c r="F1023" s="2">
+        <v>41.32</v>
+      </c>
+      <c r="G1023" s="2">
+        <v>-74.8</v>
+      </c>
+      <c r="H1023" s="2" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1024" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1024" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1024" s="2" t="s">
+        <v>1993</v>
+      </c>
+      <c r="D1024" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1024" s="2" t="s">
+        <v>1988</v>
+      </c>
+      <c r="F1024" s="2">
+        <v>41.09</v>
+      </c>
+      <c r="G1024" s="2">
+        <v>-75</v>
+      </c>
+      <c r="H1024" s="2" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1025" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1025" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1025" s="2" t="s">
+        <v>1992</v>
+      </c>
+      <c r="D1025" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1025" s="2" t="s">
+        <v>1988</v>
+      </c>
+      <c r="F1025" s="2">
+        <v>41.22</v>
+      </c>
+      <c r="G1025" s="2">
+        <v>-74.87</v>
+      </c>
+      <c r="H1025" s="2" t="s">
+        <v>1991</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:8" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1026" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1026" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1026" s="2" t="s">
+        <v>1994</v>
+      </c>
+      <c r="D1026" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1026" s="2" t="s">
+        <v>1995</v>
+      </c>
+      <c r="F1026" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1026" s="2" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:8" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1027" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1027" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1027" s="2" t="s">
+        <v>1997</v>
+      </c>
+      <c r="D1027" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1027" s="2" t="s">
+        <v>1998</v>
+      </c>
+      <c r="F1027" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1027" s="2" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:8" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1028" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1028" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1028" s="2" t="s">
+        <v>1997</v>
+      </c>
+      <c r="D1028" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1028" s="2" t="s">
+        <v>1999</v>
+      </c>
+      <c r="F1028" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1028" s="2" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:8" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1029" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1029" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1029" s="2" t="s">
+        <v>2000</v>
+      </c>
+      <c r="D1029" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1029" s="2" t="s">
+        <v>2001</v>
+      </c>
+      <c r="F1029" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1029" s="2" t="s">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:8" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1030" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1030" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1030" s="2" t="s">
+        <v>2000</v>
+      </c>
+      <c r="D1030" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1030" s="2" t="s">
+        <v>2003</v>
+      </c>
+      <c r="F1030" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1030" s="2" t="s">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:8" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1031" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1031" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1031" s="2" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D1031" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1031" s="2" t="s">
+        <v>2005</v>
+      </c>
+      <c r="F1031" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1031" s="2" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:8" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1032" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1032" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1032" s="2" t="s">
+        <v>2007</v>
+      </c>
+      <c r="D1032" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1032" s="2" t="s">
+        <v>2008</v>
+      </c>
+      <c r="F1032" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1032" s="2" t="s">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:8" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1033" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1033" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1033" s="2" t="s">
+        <v>2007</v>
+      </c>
+      <c r="D1033" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1033" s="2" t="s">
+        <v>2010</v>
+      </c>
+      <c r="F1033" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1033" s="2" t="s">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:8" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1034" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1034" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1034" s="2" t="s">
+        <v>2011</v>
+      </c>
+      <c r="D1034" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1034" s="2" t="s">
+        <v>2012</v>
+      </c>
+      <c r="F1034" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1034" s="2" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A1035" s="2" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1035" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1035" s="2" t="s">
+        <v>2014</v>
+      </c>
+      <c r="D1035" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1035" s="2" t="s">
+        <v>2015</v>
+      </c>
+      <c r="F1035" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1035" s="2" t="s">
+        <v>2016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>